<commit_message>
hw06: record A-AI-035 lockout-expiry as a manual FAILED run (BUG-04)
The 30-second lockout-expiry case was executed manually with a timed wait and
returned 403 (still locked): the SUT locks ~180s instead of the spec's 30s.
Mark it executed/FAILED, fold it into BUG-04, and update counts to 120 executed,
47 passed, 73 failed, 0 not run.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017raCYLezV1Teg5XKx4GohA
</commit_message>
<xml_diff>
--- a/HW06-AI/reports/23127272_HW06_test_cases.xlsx
+++ b/HW06-AI/reports/23127272_HW06_test_cases.xlsx
@@ -3687,11 +3687,19 @@
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>NOT RUN</t>
-        </is>
-      </c>
-      <c r="O36" s="2" t="inlineStr"/>
-      <c r="P36" s="2" t="inlineStr"/>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>403</t>
+        </is>
+      </c>
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>Manually executed with a 30-second wait; the account was still locked (HTTP 403). The SUT locks for 180s, not the 30s the spec requires.</t>
+        </is>
+      </c>
       <c r="Q36" s="2" t="inlineStr"/>
       <c r="R36" s="2" t="inlineStr">
         <is>
@@ -11500,7 +11508,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C5" t="n">
         <v>40</v>
@@ -11509,7 +11517,7 @@
         <v>40</v>
       </c>
       <c r="E5" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6">
@@ -11538,7 +11546,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C7" t="n">
         <v>26</v>
@@ -11547,7 +11555,7 @@
         <v>26</v>
       </c>
       <c r="E7" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8">
@@ -11557,7 +11565,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C8" t="n">
         <v>0</v>
@@ -11566,7 +11574,7 @@
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">

</xml_diff>